<commit_message>
increased cubed dims in high_dim_con
</commit_message>
<xml_diff>
--- a/high_dim_con.xlsx
+++ b/high_dim_con.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/srinath/Documents/GitHub/cuda_python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A0FF6FD-A6C2-A047-A920-EEA3EA945289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9A52115-9EE1-9D4C-A3E8-0D8D6ADB274C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{E3220547-C2A3-8B4E-97D6-08DE130750E0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="110">
   <si>
     <t>adim</t>
   </si>
@@ -324,6 +324,48 @@
   </si>
   <si>
     <t>(2000, 640, 200)</t>
+  </si>
+  <si>
+    <t>(300, 300)</t>
+  </si>
+  <si>
+    <t>(300, 300, 300)</t>
+  </si>
+  <si>
+    <t>(300, 300 300)</t>
+  </si>
+  <si>
+    <t>([2], [2])</t>
+  </si>
+  <si>
+    <t>(300, 300, 300, 300)</t>
+  </si>
+  <si>
+    <t>(100, 100, 100)</t>
+  </si>
+  <si>
+    <t>(100, 100, 100, 100)</t>
+  </si>
+  <si>
+    <t>(100, 100)</t>
+  </si>
+  <si>
+    <t>(600, 600, 600)</t>
+  </si>
+  <si>
+    <t>(600, 600, 600, 600)</t>
+  </si>
+  <si>
+    <t>(600, 600)</t>
+  </si>
+  <si>
+    <t>(50, 50, 50)</t>
+  </si>
+  <si>
+    <t>(50, 50, 50, 50)</t>
+  </si>
+  <si>
+    <t>(50, 50)</t>
   </si>
 </sst>
 </file>
@@ -390,12 +432,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -710,7 +754,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{533FA1DA-7CC0-DB47-8E54-9F4B65E35022}">
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.1640625" customWidth="1"/>
@@ -2031,6 +2075,374 @@
         <v>47</v>
       </c>
     </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>97</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G58" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>97</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>101</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G60" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>101</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C61" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G61" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A62" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A63" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G63" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>107</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G64" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A65" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G65" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>96</v>
+      </c>
+      <c r="B66" t="s">
+        <v>96</v>
+      </c>
+      <c r="C66" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>96</v>
+      </c>
+      <c r="B67" t="s">
+        <v>96</v>
+      </c>
+      <c r="C67" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>103</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>103</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>106</v>
+      </c>
+      <c r="B70" t="s">
+        <v>106</v>
+      </c>
+      <c r="C70" t="s">
+        <v>106</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>106</v>
+      </c>
+      <c r="B71" t="s">
+        <v>106</v>
+      </c>
+      <c r="C71" t="s">
+        <v>106</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>109</v>
+      </c>
+      <c r="B72" t="s">
+        <v>109</v>
+      </c>
+      <c r="C72" t="s">
+        <v>109</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>109</v>
+      </c>
+      <c r="B73" t="s">
+        <v>109</v>
+      </c>
+      <c r="C73" t="s">
+        <v>109</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated removed huge contraction
</commit_message>
<xml_diff>
--- a/high_dim_con.xlsx
+++ b/high_dim_con.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/srinath/Documents/GitHub/cuda_python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC23779F-A35F-0444-8755-4CF2CF76E7D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B778539F-9220-7C43-AD8F-9263F3A732F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{E3220547-C2A3-8B4E-97D6-08DE130750E0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="107">
   <si>
     <t>adim</t>
   </si>
@@ -345,12 +345,6 @@
   </si>
   <si>
     <t>(100, 100)</t>
-  </si>
-  <si>
-    <t>(600, 600, 600)</t>
-  </si>
-  <si>
-    <t>(600, 600, 600, 600)</t>
   </si>
   <si>
     <t>(600, 600)</t>
@@ -751,7 +745,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{533FA1DA-7CC0-DB47-8E54-9F4B65E35022}">
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.1640625" customWidth="1"/>
@@ -2165,14 +2159,14 @@
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A62" s="4" t="s">
-        <v>103</v>
+      <c r="A62" t="s">
+        <v>104</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>98</v>
@@ -2189,13 +2183,13 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D63" s="1" t="s">
         <v>98</v>
@@ -2212,59 +2206,59 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>106</v>
-      </c>
-      <c r="B64" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C64" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E64" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F64" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G64" s="4" t="s">
-        <v>24</v>
+        <v>96</v>
+      </c>
+      <c r="B64" t="s">
+        <v>96</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A65" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="B65" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C65" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E65" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G65" s="4" t="s">
-        <v>26</v>
+      <c r="A65" t="s">
+        <v>96</v>
+      </c>
+      <c r="B65" t="s">
+        <v>96</v>
+      </c>
+      <c r="C65" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>96</v>
-      </c>
-      <c r="B66" t="s">
-        <v>96</v>
-      </c>
-      <c r="C66" s="5" t="s">
-        <v>96</v>
+        <v>102</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>102</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>28</v>
@@ -2281,13 +2275,13 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>96</v>
-      </c>
-      <c r="B67" t="s">
-        <v>96</v>
-      </c>
-      <c r="C67" s="5" t="s">
-        <v>96</v>
+        <v>102</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>102</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>28</v>
@@ -2304,13 +2298,13 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>102</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
+      </c>
+      <c r="B68" t="s">
+        <v>103</v>
+      </c>
+      <c r="C68" t="s">
+        <v>103</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>28</v>
@@ -2327,13 +2321,13 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>102</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
+      </c>
+      <c r="B69" t="s">
+        <v>103</v>
+      </c>
+      <c r="C69" t="s">
+        <v>103</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>28</v>
@@ -2350,13 +2344,13 @@
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B70" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C70" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>28</v>
@@ -2373,13 +2367,13 @@
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B71" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C71" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>28</v>
@@ -2391,52 +2385,6 @@
         <v>20</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
-        <v>108</v>
-      </c>
-      <c r="B72" t="s">
-        <v>108</v>
-      </c>
-      <c r="C72" t="s">
-        <v>108</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F72" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G72" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
-        <v>108</v>
-      </c>
-      <c r="B73" t="s">
-        <v>108</v>
-      </c>
-      <c r="C73" t="s">
-        <v>108</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E73" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G73" s="2" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>